<commit_message>
Actualiza y regenera excels individuales/master, y documenta fix para electivos de musica
</commit_message>
<xml_diff>
--- a/bases de datos planes y programas/planes_ciencias_naturales.xlsx
+++ b/bases de datos planes y programas/planes_ciencias_naturales.xlsx
@@ -1,15 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planes Curriculares" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Planes Curriculares" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Planes Curriculares'!$A$1:$G$178</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -469,12 +471,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="64" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -522,7 +524,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -569,7 +571,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -611,7 +613,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -652,7 +654,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -692,7 +694,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -733,7 +735,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -775,7 +777,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -820,7 +822,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -865,7 +867,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -907,7 +909,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -949,7 +951,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -991,7 +993,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -1032,7 +1034,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1074,7 +1076,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -1115,7 +1117,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1155,7 +1157,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1194,7 +1196,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1235,7 +1237,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1277,7 +1279,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1317,7 +1319,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1358,7 +1360,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1398,7 +1400,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1440,7 +1442,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1482,7 +1484,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -1523,7 +1525,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1566,7 +1568,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -1607,7 +1609,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1648,7 +1650,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -1691,7 +1693,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1732,7 +1734,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -1774,7 +1776,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1815,7 +1817,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -1855,7 +1857,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1894,7 +1896,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
@@ -1934,7 +1936,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1974,7 +1976,7 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -2016,7 +2018,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2055,7 +2057,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -2101,7 +2103,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2143,7 +2145,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -2186,7 +2188,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2229,7 +2231,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
@@ -2271,7 +2273,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2310,7 +2312,7 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -2352,7 +2354,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2393,7 +2395,7 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -2436,7 +2438,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -2477,7 +2479,7 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
@@ -2520,7 +2522,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -2561,7 +2563,7 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -2602,7 +2604,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -2641,7 +2643,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -2679,7 +2681,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -2718,7 +2720,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
@@ -2760,7 +2762,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -2801,7 +2803,7 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
@@ -2842,7 +2844,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -2882,7 +2884,7 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -2923,7 +2925,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -2962,7 +2964,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -3001,7 +3003,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -3042,7 +3044,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -3081,7 +3083,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -3124,7 +3126,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -3167,7 +3169,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -3209,7 +3211,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
@@ -3251,7 +3253,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -3293,7 +3295,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
@@ -3332,7 +3334,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -3372,7 +3374,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -3414,7 +3416,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -3454,7 +3456,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -3494,7 +3496,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -3535,7 +3537,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
@@ -3574,7 +3576,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3612,7 +3614,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
@@ -3651,7 +3653,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -3692,7 +3694,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
@@ -3733,7 +3735,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -3775,7 +3777,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
@@ -3817,7 +3819,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -3859,7 +3861,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
@@ -3904,7 +3906,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -3945,7 +3947,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
@@ -3988,7 +3990,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -4029,7 +4031,7 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
@@ -4070,7 +4072,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -4111,7 +4113,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
@@ -4151,7 +4153,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -4193,7 +4195,7 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
@@ -4234,7 +4236,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -4274,7 +4276,7 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
@@ -4316,7 +4318,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -4357,7 +4359,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
@@ -4397,7 +4399,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -4436,7 +4438,7 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
@@ -4474,7 +4476,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -4517,7 +4519,7 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
@@ -4557,7 +4559,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -4599,7 +4601,7 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
@@ -4640,7 +4642,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -4682,7 +4684,7 @@
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
@@ -4724,7 +4726,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -4764,7 +4766,7 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
@@ -4808,7 +4810,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -4850,7 +4852,7 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
@@ -4890,7 +4892,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -4933,7 +4935,7 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
@@ -4977,7 +4979,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -5017,7 +5019,7 @@
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
@@ -5057,7 +5059,7 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -5098,7 +5100,7 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
@@ -5139,7 +5141,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -5182,7 +5184,7 @@
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
@@ -5225,7 +5227,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -5266,7 +5268,7 @@
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
@@ -5308,7 +5310,7 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -5351,7 +5353,7 @@
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
@@ -5392,7 +5394,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
@@ -5436,7 +5438,7 @@
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
@@ -5478,7 +5480,7 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
@@ -5523,7 +5525,7 @@
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
@@ -5565,7 +5567,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -5605,7 +5607,7 @@
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
@@ -5646,7 +5648,7 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -5686,7 +5688,7 @@
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
@@ -5727,7 +5729,7 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
@@ -5767,7 +5769,7 @@
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
@@ -5809,7 +5811,7 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
@@ -5852,7 +5854,7 @@
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
@@ -5893,7 +5895,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -5936,7 +5938,7 @@
       </c>
       <c r="B133" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
@@ -5979,7 +5981,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -6022,7 +6024,7 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
@@ -6066,7 +6068,7 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -6112,7 +6114,7 @@
       </c>
       <c r="B137" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
@@ -6156,7 +6158,7 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
@@ -6198,7 +6200,7 @@
       </c>
       <c r="B139" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
@@ -6239,7 +6241,7 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
@@ -6279,7 +6281,7 @@
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
@@ -6321,7 +6323,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -6366,7 +6368,7 @@
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
@@ -6407,7 +6409,7 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -6451,7 +6453,7 @@
       </c>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
@@ -6493,7 +6495,7 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
@@ -6536,7 +6538,7 @@
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
@@ -6578,7 +6580,7 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -6621,7 +6623,7 @@
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C149" s="5" t="inlineStr">
@@ -6663,7 +6665,7 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
@@ -6708,7 +6710,7 @@
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C151" s="5" t="inlineStr">
@@ -6752,7 +6754,7 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
@@ -6796,7 +6798,7 @@
       </c>
       <c r="B153" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
@@ -6841,7 +6843,7 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
@@ -6882,7 +6884,7 @@
       </c>
       <c r="B155" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C155" s="5" t="inlineStr">
@@ -6925,7 +6927,7 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
@@ -6967,7 +6969,7 @@
       </c>
       <c r="B157" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C157" s="5" t="inlineStr">
@@ -7009,7 +7011,7 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
@@ -7051,7 +7053,7 @@
       </c>
       <c r="B159" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C159" s="5" t="inlineStr">
@@ -7093,7 +7095,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
@@ -7136,7 +7138,7 @@
       </c>
       <c r="B161" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C161" s="5" t="inlineStr">
@@ -7179,7 +7181,7 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
@@ -7220,7 +7222,7 @@
       </c>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C163" s="5" t="inlineStr">
@@ -7261,7 +7263,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
@@ -7302,7 +7304,7 @@
       </c>
       <c r="B165" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C165" s="5" t="inlineStr">
@@ -7345,7 +7347,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
@@ -7388,7 +7390,7 @@
       </c>
       <c r="B167" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C167" s="5" t="inlineStr">
@@ -7429,7 +7431,7 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
@@ -7471,7 +7473,7 @@
       </c>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C169" s="5" t="inlineStr">
@@ -7514,7 +7516,7 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
@@ -7556,7 +7558,7 @@
       </c>
       <c r="B171" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C171" s="5" t="inlineStr">
@@ -7598,7 +7600,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
@@ -7641,7 +7643,7 @@
       </c>
       <c r="B173" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C173" s="5" t="inlineStr">
@@ -7683,7 +7685,7 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
@@ -7724,7 +7726,7 @@
       </c>
       <c r="B175" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C175" s="5" t="inlineStr">
@@ -7766,7 +7768,7 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
@@ -7808,7 +7810,7 @@
       </c>
       <c r="B177" s="4" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C177" s="5" t="inlineStr">
@@ -7851,7 +7853,7 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Ciencias naturales</t>
+          <t>Ciencias Naturales</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
@@ -7887,6 +7889,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G178"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>